<commit_message>
added one number for data articles text from Blanka; rendered index.
</commit_message>
<xml_diff>
--- a/archive/DCC archiving information/archiving_files_that_were_created_in_archived_scripts.xlsx
+++ b/archive/DCC archiving information/archiving_files_that_were_created_in_archived_scripts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AVIHAY\git\DCC-v3\archive\DCC archiving information\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9312F5D-AE8B-4FA8-8E29-85C812A8030D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79D62534-BD1B-4CE8-A4B9-3A21B05009D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19080" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -612,121 +612,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="15">
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill patternType="none">
@@ -2610,7 +2496,7 @@
     </sortState>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="C2:E70">
-    <sortCondition sortBy="cellColor" ref="C2:C70" dxfId="14"/>
+    <sortCondition sortBy="cellColor" ref="C2:C70" dxfId="0"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>